<commit_message>
SEO sheet: include location in keyphrase, title and description
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LVXsfLowwpctuiRtH2tMVR
</commit_message>
<xml_diff>
--- a/creem-llar/output/seo-creem-llar.xlsx
+++ b/creem-llar/output/seo-creem-llar.xlsx
@@ -502,27 +502,27 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>estudi d'interiorisme Figueres</t>
+          <t>estudi d'interiorisme a Figueres</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Estudi d'interiorisme Figueres | Cuines, banys i reformes</t>
+          <t>Estudi d'interiorisme a Figueres | Cuines, banys i reformes</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>500</v>
+        <v>517</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Estudi d'interiorisme Figueres i Banyoles: dissenyem cuines, banys, reformes i parquets a mida per crear llars úniques. Demana pressupost sense compromís.</t>
+          <t>Estudi d'interiorisme a Figueres i Banyoles: dissenyem cuines, banys, reformes i parquets a mida per crear llars úniques. Demana pressupost sense compromís.</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -543,19 +543,19 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>projectes d'interiorisme</t>
+          <t>projectes d'interiorisme a l'Empordà</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Projectes d'interiorisme | Cuines, banys i reformes Girona</t>
+          <t>Projectes d'interiorisme a l'Empordà | Creem Llar Figueres</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
         <v>58</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>510</v>
+        <v>517</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -584,27 +584,27 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>cuines a mida Figueres</t>
+          <t>cuines a Figueres</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Cuines a mida Figueres | Disseny i muntatge – Creem Llar</t>
+          <t>Cuines a Figueres | Disseny a mida i muntatge – Creem Llar</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>519</v>
+        <v>535</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Cuines a mida Figueres i Banyoles: dissenys funcionals i elegants per al teu dia a dia, amb materials de qualitat i acompanyament total. Demana pressupost.</t>
+          <t>Cuines a Figueres i Banyoles: dissenys a mida funcionals i elegants per al teu dia a dia, amb materials de qualitat i acompanyament. Demana pressupost.</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -625,27 +625,27 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>reformes de banys Banyoles</t>
+          <t>banys a Banyoles</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Reformes de banys Banyoles | Espais moderns – Creem Llar</t>
+          <t>Banys a Banyoles | Reformes de banys a mida – Creem Llar</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
         <v>56</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>542</v>
+        <v>537</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Reformes de banys Banyoles i Figueres: espais moderns, còmodes i plens de benestar, amb disseny a mida i garantia. Explica'ns la teva idea sense compromís.</t>
+          <t>Banys a Banyoles i Figueres: reformes d'espais moderns, còmodes i plens de benestar, amb disseny a mida i garantia. Explica'ns la teva idea sense compromís.</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -666,27 +666,27 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>disseny d'interiors a mida</t>
+          <t>disseny d'interiors a Banyoles</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Disseny d'interiors a mida | Interiorisme Figueres – Creem Llar</t>
+          <t>Disseny d'interiors a Banyoles | Creem Llar Figueres</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>554</v>
+        <v>466</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Disseny d'interiors a mida per a cada estil de vida: combinem estètica, funcionalitat i benestar a Figueres i Banyoles. Parla amb el nostre equip.</t>
+          <t>Disseny d'interiors a Banyoles i Figueres per a cada estil de vida: combinem estètica, funcionalitat i benestar. Parla amb el nostre equip d'interioristes.</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
-        <v>146</v>
+        <v>155</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
@@ -712,14 +712,14 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Parquets a Figueres | Paviments càlids per a la teva llar</t>
+          <t>Parquets a Figueres i Banyoles | Paviments càlids per a la llar</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>494</v>
+        <v>549</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
@@ -748,27 +748,27 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>equip d'interioristes Figueres</t>
+          <t>equip d'interioristes a Figueres</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Equip d'interioristes Figueres | Qui som – Creem Llar</t>
+          <t>Equip d'interioristes a Figueres | Qui som – Creem Llar</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>469</v>
+        <v>486</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Equip d'interioristes Figueres: Carlos, Xavi i Samuel lideren un equip de professionals que dissenya i executa espais per viure, fins a l'últim detall.</t>
+          <t>Equip d'interioristes a Figueres: Carlos, Xavi i Samuel lideren un equip de professionals que dissenya i executa espais per viure, fins a l'últim detall.</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -789,27 +789,27 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>pressupost de reformes</t>
+          <t>pressupost de reformes Figueres</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Pressupost de reformes | Contacta amb Creem Llar a Girona</t>
+          <t>Pressupost de reformes Figueres | Contacta amb Creem Llar</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
         <v>57</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Pressupost de reformes a Figueres i Banyoles sense compromís: truca al 972 684 896 o 972 519 324, o escriu-nos a info@creemllar.com i t'assessorem.</t>
+          <t>Pressupost de reformes Figueres i Banyoles sense compromís: truca al 972 684 896 o 972 519 324, o escriu-nos a info@creemllar.com i t'assessorem.</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>

</xml_diff>